<commit_message>
feat: upgrade god-tier rating and secure PDPA compliance
</commit_message>
<xml_diff>
--- a/อสม.xlsx
+++ b/อสม.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>เลขประจำตัวประชาชน</t>
   </si>
@@ -132,9 +132,6 @@
     <t>นาง จรรยา ค่ำสุริยา</t>
   </si>
   <si>
-    <t>นาง สำลี เชื้อดี</t>
-  </si>
-  <si>
     <t>นาง ลัดดาวัลย์ โสกขุนทด</t>
   </si>
   <si>
@@ -190,6 +187,18 @@
   </si>
   <si>
     <t>นางสาวสุรินทร์ญา เพชร์หงษ์</t>
+  </si>
+  <si>
+    <t>นาง ศุภากร เชื้อดี</t>
+  </si>
+  <si>
+    <t>นางวิชชุดา กอนแสง</t>
+  </si>
+  <si>
+    <t>นางสาวแสงดาว กงแก้ว</t>
+  </si>
+  <si>
+    <t>นายสิรภพ แก้วทิพย์</t>
   </si>
 </sst>
 </file>
@@ -530,10 +539,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.75" style="1" customWidth="1"/>
+    <col min="1" max="1" width="19.375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -837,7 +846,7 @@
         <v>3251000432397</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
@@ -845,7 +854,7 @@
         <v>3251000433458</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
@@ -853,7 +862,7 @@
         <v>3251000432176</v>
       </c>
       <c r="B40" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
@@ -861,7 +870,7 @@
         <v>3251000435442</v>
       </c>
       <c r="B41" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
@@ -869,7 +878,7 @@
         <v>3251000436392</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
@@ -877,7 +886,7 @@
         <v>2251000016344</v>
       </c>
       <c r="B43" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
@@ -885,7 +894,7 @@
         <v>3251000435230</v>
       </c>
       <c r="B44" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
@@ -893,7 +902,7 @@
         <v>3251000440578</v>
       </c>
       <c r="B45" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
@@ -901,7 +910,7 @@
         <v>3251000434870</v>
       </c>
       <c r="B46" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
@@ -909,7 +918,7 @@
         <v>3251000012371</v>
       </c>
       <c r="B47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
@@ -917,7 +926,7 @@
         <v>3251000434977</v>
       </c>
       <c r="B48" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -925,7 +934,7 @@
         <v>3251000436422</v>
       </c>
       <c r="B49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
@@ -933,7 +942,7 @@
         <v>3160300818193</v>
       </c>
       <c r="B50" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
@@ -941,7 +950,7 @@
         <v>3251000439421</v>
       </c>
       <c r="B51" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
@@ -949,7 +958,7 @@
         <v>5251099004445</v>
       </c>
       <c r="B52" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
@@ -957,7 +966,7 @@
         <v>3251000435485</v>
       </c>
       <c r="B53" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
@@ -965,7 +974,7 @@
         <v>1279800001715</v>
       </c>
       <c r="B54" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
@@ -973,7 +982,7 @@
         <v>1409800066521</v>
       </c>
       <c r="B55" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
@@ -981,7 +990,7 @@
         <v>1100200918351</v>
       </c>
       <c r="B56" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
@@ -989,11 +998,36 @@
         <v>3251000432213</v>
       </c>
       <c r="B57" t="s">
-        <v>57</v>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" s="1">
+        <v>3251000441639</v>
+      </c>
+      <c r="B58" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" s="1">
+        <v>1259700107058</v>
+      </c>
+      <c r="B59" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="1">
+        <v>1279800022828</v>
+      </c>
+      <c r="B60" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>